<commit_message>
correciones a correlaciones de pearson y ajuste para conteos de episodios de ENOS
</commit_message>
<xml_diff>
--- a/CODIGOS/CONTEO/conteo_ENSO_por_año.xlsx
+++ b/CODIGOS/CONTEO/conteo_ENSO_por_año.xlsx
@@ -449,7 +449,7 @@
         <v>1951</v>
       </c>
       <c r="B3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C3" t="n">
         <v>1</v>
@@ -460,10 +460,10 @@
         <v>1952</v>
       </c>
       <c r="B4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5">
@@ -471,7 +471,7 @@
         <v>1953</v>
       </c>
       <c r="B5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C5" t="n">
         <v>0</v>
@@ -482,7 +482,7 @@
         <v>1954</v>
       </c>
       <c r="B6" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C6" t="n">
         <v>1</v>
@@ -526,7 +526,7 @@
         <v>1958</v>
       </c>
       <c r="B10" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C10" t="n">
         <v>0</v>
@@ -537,10 +537,10 @@
         <v>1959</v>
       </c>
       <c r="B11" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C11" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="12">
@@ -551,7 +551,7 @@
         <v>0</v>
       </c>
       <c r="C12" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="13">
@@ -573,7 +573,7 @@
         <v>0</v>
       </c>
       <c r="C14" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="15">
@@ -628,7 +628,7 @@
         <v>0</v>
       </c>
       <c r="C19" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="20">
@@ -636,7 +636,7 @@
         <v>1968</v>
       </c>
       <c r="B20" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C20" t="n">
         <v>1</v>
@@ -647,7 +647,7 @@
         <v>1969</v>
       </c>
       <c r="B21" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="C21" t="n">
         <v>0</v>
@@ -658,7 +658,7 @@
         <v>1970</v>
       </c>
       <c r="B22" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C22" t="n">
         <v>1</v>
@@ -724,7 +724,7 @@
         <v>1976</v>
       </c>
       <c r="B28" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C28" t="n">
         <v>1</v>
@@ -735,7 +735,7 @@
         <v>1977</v>
       </c>
       <c r="B29" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="C29" t="n">
         <v>0</v>
@@ -746,7 +746,7 @@
         <v>1978</v>
       </c>
       <c r="B30" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C30" t="n">
         <v>1</v>
@@ -757,10 +757,10 @@
         <v>1979</v>
       </c>
       <c r="B31" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C31" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="32">
@@ -768,7 +768,7 @@
         <v>1980</v>
       </c>
       <c r="B32" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C32" t="n">
         <v>0</v>
@@ -782,7 +782,7 @@
         <v>0</v>
       </c>
       <c r="C33" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="34">
@@ -804,7 +804,7 @@
         <v>1</v>
       </c>
       <c r="C35" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="36">
@@ -837,7 +837,7 @@
         <v>1</v>
       </c>
       <c r="C38" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="39">
@@ -878,7 +878,7 @@
         <v>1990</v>
       </c>
       <c r="B42" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C42" t="n">
         <v>0</v>
@@ -911,7 +911,7 @@
         <v>1993</v>
       </c>
       <c r="B45" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="C45" t="n">
         <v>0</v>
@@ -922,7 +922,7 @@
         <v>1994</v>
       </c>
       <c r="B46" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C46" t="n">
         <v>0</v>
@@ -933,7 +933,7 @@
         <v>1995</v>
       </c>
       <c r="B47" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C47" t="n">
         <v>1</v>
@@ -958,7 +958,7 @@
         <v>1</v>
       </c>
       <c r="C49" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="50">
@@ -991,7 +991,7 @@
         <v>0</v>
       </c>
       <c r="C52" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="53">
@@ -1013,7 +1013,7 @@
         <v>1</v>
       </c>
       <c r="C54" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="55">
@@ -1021,7 +1021,7 @@
         <v>2003</v>
       </c>
       <c r="B55" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C55" t="n">
         <v>0</v>
@@ -1046,7 +1046,7 @@
         <v>1</v>
       </c>
       <c r="C57" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="58">
@@ -1054,10 +1054,10 @@
         <v>2006</v>
       </c>
       <c r="B58" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C58" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="59">
@@ -1065,7 +1065,7 @@
         <v>2007</v>
       </c>
       <c r="B59" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C59" t="n">
         <v>1</v>
@@ -1090,7 +1090,7 @@
         <v>1</v>
       </c>
       <c r="C61" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="62">
@@ -1112,7 +1112,7 @@
         <v>0</v>
       </c>
       <c r="C63" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="64">
@@ -1120,10 +1120,10 @@
         <v>2012</v>
       </c>
       <c r="B64" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C64" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="65">
@@ -1134,7 +1134,7 @@
         <v>0</v>
       </c>
       <c r="C65" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="66">
@@ -1142,10 +1142,10 @@
         <v>2014</v>
       </c>
       <c r="B66" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C66" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="67">
@@ -1167,7 +1167,7 @@
         <v>1</v>
       </c>
       <c r="C68" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="69">
@@ -1178,7 +1178,7 @@
         <v>0</v>
       </c>
       <c r="C69" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="70">

</xml_diff>